<commit_message>
Resolved conflicts by keeping main versions of data and Rproj
</commit_message>
<xml_diff>
--- a/oasis_cross-sectional-5708aa0a98d82080.xlsx
+++ b/oasis_cross-sectional-5708aa0a98d82080.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maximamertens/Desktop/UvA ResMas/PIPS/PIPS_project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amsuni-my.sharepoint.com/personal/julia_stolwijk_student_uva_nl/Documents/r_course/PIPS_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{10F70CD0-899F-0144-AFE0-1C91F546456D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEBC238B-C63C-BB45-89D0-7037150F1AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="620" windowWidth="28800" windowHeight="16100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="oasis_cross-sectional" sheetId="1" r:id="rId1"/>

</xml_diff>